<commit_message>
mais uma vez correcoes
</commit_message>
<xml_diff>
--- a/Estudando/excel/modelo_relacional.xlsx
+++ b/Estudando/excel/modelo_relacional.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,11 +432,6 @@
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -451,10 +446,9 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -469,10 +463,9 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>email_field</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -487,10 +480,9 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>password</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -505,10 +497,9 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -523,10 +514,9 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -541,10 +531,9 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>email_field</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -559,10 +548,9 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -577,10 +565,9 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -595,10 +582,9 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -613,10 +599,9 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -631,10 +616,9 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -649,10 +633,9 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -667,10 +650,9 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -685,10 +667,9 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>date</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -703,10 +684,9 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -721,10 +701,9 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>url</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -739,10 +718,9 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>url</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -757,10 +735,9 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -775,10 +752,9 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
+          <t>email_field</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -793,10 +769,9 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -811,10 +786,9 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -829,10 +803,9 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -847,10 +820,9 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -865,10 +837,9 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -883,10 +854,9 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -901,10 +871,9 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>email_field</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -919,10 +888,9 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -937,10 +905,9 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -955,10 +922,9 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -973,10 +939,9 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -991,10 +956,9 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>email_field</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1009,10 +973,9 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1027,10 +990,9 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1045,10 +1007,9 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1063,10 +1024,9 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1081,10 +1041,9 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1099,10 +1058,9 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1117,10 +1075,9 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>